<commit_message>
docs(core): A5 node review and audit fixes [codex]
</commit_message>
<xml_diff>
--- a/out/evidence.xlsx
+++ b/out/evidence.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Транзакции-основания'!$A$1:$E$497</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Пути денег'!$A$1:$I$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Критерии'!$A$1:$E$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Границы данных'!$A$1:$D$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Границы данных'!$A$1:$D$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>0.7770317090554368</v>
+        <v>0.7771240025487456</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.7377590653313123</v>
+        <v>0.7378513588246211</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0.7376812614648389</v>
+        <v>0.7377735549581477</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.6851303003513609</v>
+        <v>0.6852225938446697</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.6832391542907629</v>
+        <v>0.6833314477840716</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.6815736102192874</v>
+        <v>0.6816659037125961</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.6801690391459074</v>
+        <v>0.6802613326392162</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.6741452815251672</v>
+        <v>0.6742375750184759</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>0.6633318505338077</v>
+        <v>0.6634241440271165</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.647905884038645</v>
+        <v>0.6479981775319537</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>0.6389582945730743</v>
+        <v>0.639050588066383</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.6381316725978647</v>
+        <v>0.6382239660911735</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0.6346734982918394</v>
+        <v>0.6347657917851481</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.623420818505338</v>
+        <v>0.6235131119986468</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -1131,7 +1131,7 @@
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.6116761476934649</v>
+        <v>0.6117684411867736</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.6096607126141557</v>
+        <v>0.6097530061074644</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>0.6088575815202997</v>
+        <v>0.6089498750136084</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>0.6075359225971508</v>
+        <v>0.6076282160904596</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>0.6038889154611308</v>
+        <v>0.6039812089544395</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>0.5857573290804974</v>
+        <v>0.585849622573806</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0.5778499747275745</v>
+        <v>0.5779422682208832</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="D25" s="4" t="n">
-        <v>0.5694739660911735</v>
+        <v>0.5695662595844823</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="D26" s="4" t="n">
-        <v>0.5674087862748737</v>
+        <v>0.5675010797681824</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="D27" s="4" t="n">
-        <v>0.5663064649846086</v>
+        <v>0.5663987584779173</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="D28" s="4" t="n">
-        <v>0.5650015276559455</v>
+        <v>0.5650938211492542</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -1705,7 +1705,7 @@
         </is>
       </c>
       <c r="D29" s="4" t="n">
-        <v>0.5586999016302447</v>
+        <v>0.5587921951235535</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="D30" s="4" t="n">
-        <v>0.5526362300676305</v>
+        <v>0.5527285235609392</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0.5663064649846086</v>
+        <v>0.5663987584779173</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -2319,7 +2319,7 @@
         <v>0.8067170818505338</v>
       </c>
       <c r="AU2" s="4" t="n">
-        <v>0.0041532071988924</v>
+        <v>0.004614674665436</v>
       </c>
       <c r="AV2" s="4" t="n">
         <v>0.9848754448398576</v>
@@ -2360,7 +2360,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.6088575815202997</v>
+        <v>0.6089498750136084</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -2492,7 +2492,7 @@
         <v>0.9477313167259788</v>
       </c>
       <c r="AU3" s="4" t="n">
-        <v>0.0064605445316105</v>
+        <v>0.0069220119981541</v>
       </c>
       <c r="AV3" s="4" t="n">
         <v>0.9759786476868328</v>
@@ -2533,7 +2533,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0.6633318505338077</v>
+        <v>0.6634241440271165</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -2669,7 +2669,7 @@
         <v>0.7653469750889679</v>
       </c>
       <c r="AU4" s="4" t="n">
-        <v>0</v>
+        <v>0.0004614674665436</v>
       </c>
       <c r="AV4" s="4" t="n">
         <v>0.9372775800711745</v>
@@ -2887,7 +2887,7 @@
         <v>66</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.5526362300676305</v>
+        <v>0.5527285235609392</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
         <v>0.7955960854092526</v>
       </c>
       <c r="AU6" s="4" t="n">
-        <v>0.0004614674665436</v>
+        <v>0.0009229349330872</v>
       </c>
       <c r="AV6" s="4" t="n">
         <v>0.8269572953736655</v>
@@ -3237,7 +3237,7 @@
         <v>2</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.5674087862748737</v>
+        <v>0.5675010797681824</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -3369,7 +3369,7 @@
         <v>0.9724199288256228</v>
       </c>
       <c r="AU8" s="4" t="n">
-        <v>0.0009229349330872</v>
+        <v>0.0013844023996308</v>
       </c>
       <c r="AV8" s="4" t="n">
         <v>0.854982206405694</v>
@@ -3410,7 +3410,7 @@
         <v>12</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.7377590653313123</v>
+        <v>0.7378513588246211</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -3542,7 +3542,7 @@
         <v>0.9972197508896796</v>
       </c>
       <c r="AU9" s="4" t="n">
-        <v>0.002307337332718</v>
+        <v>0.0027688047992616</v>
       </c>
       <c r="AV9" s="4" t="n">
         <v>0.9813167259786476</v>
@@ -3583,7 +3583,7 @@
         <v>13</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0.6038889154611308</v>
+        <v>0.6039812089544395</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -3715,7 +3715,7 @@
         <v>0.9164813167259788</v>
       </c>
       <c r="AU10" s="4" t="n">
-        <v>0.0041532071988924</v>
+        <v>0.004614674665436</v>
       </c>
       <c r="AV10" s="4" t="n">
         <v>0.7811387900355872</v>
@@ -3756,7 +3756,7 @@
         <v>3</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.623420818505338</v>
+        <v>0.6235131119986468</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -3892,7 +3892,7 @@
         <v>0.9695284697508896</v>
       </c>
       <c r="AU11" s="4" t="n">
-        <v>0</v>
+        <v>0.0004614674665436</v>
       </c>
       <c r="AV11" s="4" t="n">
         <v>0.8256227758007118</v>
@@ -4106,7 +4106,7 @@
         <v>12</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.6096607126141557</v>
+        <v>0.6097530061074644</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -4242,7 +4242,7 @@
         <v>0.9059163701067616</v>
       </c>
       <c r="AU13" s="4" t="n">
-        <v>0.0041532071988924</v>
+        <v>0.004614674665436</v>
       </c>
       <c r="AV13" s="4" t="n">
         <v>0.8705516014234875</v>
@@ -4283,7 +4283,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0.6741452815251672</v>
+        <v>0.6742375750184759</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -4419,7 +4419,7 @@
         <v>0.7637900355871886</v>
       </c>
       <c r="AU14" s="4" t="n">
-        <v>0.0032302722658052</v>
+        <v>0.0036917397323488</v>
       </c>
       <c r="AV14" s="4" t="n">
         <v>0.9030249110320284</v>
@@ -4460,7 +4460,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.6346734982918394</v>
+        <v>0.6347657917851481</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -4592,7 +4592,7 @@
         <v>0.7685720640569396</v>
       </c>
       <c r="AU15" s="4" t="n">
-        <v>0.0004614674665436</v>
+        <v>0.0009229349330872</v>
       </c>
       <c r="AV15" s="4" t="n">
         <v>0.7691281138790036</v>
@@ -4633,7 +4633,7 @@
         <v>51</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.5778499747275745</v>
+        <v>0.5779422682208832</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -4769,7 +4769,7 @@
         <v>0.8173932384341637</v>
       </c>
       <c r="AU16" s="4" t="n">
-        <v>0.0009229349330872</v>
+        <v>0.0013844023996308</v>
       </c>
       <c r="AV16" s="4" t="n">
         <v>0.974644128113879</v>
@@ -4810,7 +4810,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.6815736102192874</v>
+        <v>0.6816659037125961</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -4942,7 +4942,7 @@
         <v>0.8138345195729537</v>
       </c>
       <c r="AU17" s="4" t="n">
-        <v>0.0004614674665436</v>
+        <v>0.0009229349330872</v>
       </c>
       <c r="AV17" s="4" t="n">
         <v>0.9733096085409252</v>
@@ -4983,7 +4983,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.6381316725978647</v>
+        <v>0.6382239660911735</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -5115,7 +5115,7 @@
         <v>0.6970640569395017</v>
       </c>
       <c r="AU18" s="4" t="n">
-        <v>0</v>
+        <v>0.0004614674665436</v>
       </c>
       <c r="AV18" s="4" t="n">
         <v>0.8901245551601423</v>
@@ -5156,7 +5156,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.5650015276559455</v>
+        <v>0.5650938211492542</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -5292,7 +5292,7 @@
         <v>0.8020462633451957</v>
       </c>
       <c r="AU19" s="4" t="n">
-        <v>0.0009229349330872</v>
+        <v>0.0013844023996308</v>
       </c>
       <c r="AV19" s="4" t="n">
         <v>0.8527580071174378</v>
@@ -5333,7 +5333,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.6116761476934649</v>
+        <v>0.6117684411867736</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -5465,7 +5465,7 @@
         <v>0.7545596085409252</v>
       </c>
       <c r="AU20" s="4" t="n">
-        <v>0.0018458698661744</v>
+        <v>0.002307337332718</v>
       </c>
       <c r="AV20" s="4" t="n">
         <v>0.9301601423487544</v>
@@ -5506,7 +5506,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0.6851303003513609</v>
+        <v>0.6852225938446697</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -5638,7 +5638,7 @@
         <v>0.739991103202847</v>
       </c>
       <c r="AU21" s="4" t="n">
-        <v>0.0013844023996308</v>
+        <v>0.0018458698661744</v>
       </c>
       <c r="AV21" s="4" t="n">
         <v>0.8616548042704626</v>
@@ -5679,7 +5679,7 @@
         <v>20</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>0.6832391542907629</v>
+        <v>0.6833314477840716</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -5811,7 +5811,7 @@
         <v>0.7670151245551602</v>
       </c>
       <c r="AU22" s="4" t="n">
-        <v>0.0018458698661744</v>
+        <v>0.002307337332718</v>
       </c>
       <c r="AV22" s="4" t="n">
         <v>0.9043594306049824</v>
@@ -5852,7 +5852,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.5694739660911735</v>
+        <v>0.5695662595844823</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -5988,7 +5988,7 @@
         <v>0.9690836298932384</v>
       </c>
       <c r="AU23" s="4" t="n">
-        <v>0.0004614674665436</v>
+        <v>0.0009229349330872</v>
       </c>
       <c r="AV23" s="4" t="n">
         <v>0.8865658362989324</v>
@@ -6029,7 +6029,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>0.6075359225971508</v>
+        <v>0.6076282160904596</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -6165,7 +6165,7 @@
         <v>0.9726423487544484</v>
       </c>
       <c r="AU24" s="4" t="n">
-        <v>0.0013844023996308</v>
+        <v>0.0018458698661744</v>
       </c>
       <c r="AV24" s="4" t="n">
         <v>0.939946619217082</v>
@@ -6206,7 +6206,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>0.6801690391459074</v>
+        <v>0.6802613326392162</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -6338,7 +6338,7 @@
         <v>0.8069395017793595</v>
       </c>
       <c r="AU25" s="4" t="n">
-        <v>0</v>
+        <v>0.0004614674665436</v>
       </c>
       <c r="AV25" s="4" t="n">
         <v>0.9808718861209964</v>
@@ -6379,7 +6379,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>0.5586999016302447</v>
+        <v>0.5587921951235535</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -6515,7 +6515,7 @@
         <v>0.9435053380782918</v>
       </c>
       <c r="AU26" s="4" t="n">
-        <v>0.002307337332718</v>
+        <v>0.0027688047992616</v>
       </c>
       <c r="AV26" s="4" t="n">
         <v>0.8518683274021353</v>
@@ -6556,7 +6556,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0.647905884038645</v>
+        <v>0.6479981775319537</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -6688,7 +6688,7 @@
         <v>0.7737989323843416</v>
       </c>
       <c r="AU27" s="4" t="n">
-        <v>0.0013844023996308</v>
+        <v>0.0018458698661744</v>
       </c>
       <c r="AV27" s="4" t="n">
         <v>0.7548932384341637</v>
@@ -6729,7 +6729,7 @@
         <v>3</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0.7770317090554368</v>
+        <v>0.7771240025487456</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -6865,7 +6865,7 @@
         <v>0.9283807829181494</v>
       </c>
       <c r="AU28" s="4" t="n">
-        <v>0.0041532071988924</v>
+        <v>0.004614674665436</v>
       </c>
       <c r="AV28" s="4" t="n">
         <v>0.9768683274021353</v>
@@ -6906,7 +6906,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>0.7376812614648389</v>
+        <v>0.7377735549581477</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -7042,7 +7042,7 @@
         <v>0.8002669039145907</v>
       </c>
       <c r="AU29" s="4" t="n">
-        <v>0.0004614674665436</v>
+        <v>0.0009229349330872</v>
       </c>
       <c r="AV29" s="4" t="n">
         <v>0.9750889679715302</v>
@@ -7083,7 +7083,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>0.5857573290804974</v>
+        <v>0.585849622573806</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -7219,7 +7219,7 @@
         <v>0.811943950177936</v>
       </c>
       <c r="AU30" s="4" t="n">
-        <v>0.0004614674665436</v>
+        <v>0.0009229349330872</v>
       </c>
       <c r="AV30" s="4" t="n">
         <v>0.9208185053380784</v>
@@ -7260,7 +7260,7 @@
         <v>9</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>0.6389582945730743</v>
+        <v>0.639050588066383</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -7396,7 +7396,7 @@
         <v>0.8084964412811388</v>
       </c>
       <c r="AU31" s="4" t="n">
-        <v>0.0119981541301338</v>
+        <v>0.0124596215966774</v>
       </c>
       <c r="AV31" s="4" t="n">
         <v>0.965747330960854</v>
@@ -24253,10 +24253,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="47" customWidth="1" min="4" max="4"/>
@@ -24399,16 +24399,24 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>неполная выгрузка</t>
+          <t>запрос</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>audit.csv</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
+          <t>запросить время транзакций для точного FlowTrace</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>100000008165763100</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>ранг 1: в выгрузке есть даты, но нет времени</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -24423,12 +24431,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>100000008165763100</t>
+          <t>100000003115284100</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ранг 1: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 2: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24445,12 +24453,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>100000003115284100</t>
+          <t>100000008686313100</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>ранг 2: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 3: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24467,12 +24475,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>100000008686313100</t>
+          <t>100000005339662100</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>ранг 3: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 4: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24489,12 +24497,12 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>100000005339662100</t>
+          <t>100000005527892100</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>ранг 4: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 5: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24511,12 +24519,12 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>100000005527892100</t>
+          <t>100000004299488100</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>ранг 5: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 6: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24533,12 +24541,12 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>100000004299488100</t>
+          <t>100000007055802100</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>ранг 6: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 7: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24555,12 +24563,12 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>100000007055802100</t>
+          <t>100000004070318100</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>ранг 7: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 8: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24577,12 +24585,12 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>100000004070318100</t>
+          <t>100000002398779100</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>ранг 8: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 9: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24594,7 +24602,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -24604,7 +24612,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>ранг 9: в выгрузке есть даты, но нет времени</t>
+          <t>67% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -24616,17 +24624,17 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>100000002398779100</t>
+          <t>100000008111003100</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>67% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 10: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24643,12 +24651,12 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>100000008111003100</t>
+          <t>100000008748408100</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>ранг 10: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 11: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24665,12 +24673,12 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>100000008748408100</t>
+          <t>100000004486525100</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>ранг 11: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 12: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24687,12 +24695,12 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>100000004486525100</t>
+          <t>100000004071080100</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ранг 12: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 13: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24704,7 +24712,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -24714,7 +24722,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>ранг 13: в выгрузке есть даты, но нет времени</t>
+          <t>60% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -24726,17 +24734,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>100000004071080100</t>
+          <t>100000003299365100</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>60% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 14: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24753,12 +24761,12 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>100000003299365100</t>
+          <t>100000004759121100</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>ранг 14: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 15: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24775,12 +24783,12 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>100000004759121100</t>
+          <t>100000003635170100</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>ранг 15: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 16: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24797,12 +24805,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>100000003635170100</t>
+          <t>100000001530983100</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>ранг 16: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 17: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24819,12 +24827,12 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>100000001530983100</t>
+          <t>100000006518161100</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>ранг 17: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 18: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24841,12 +24849,12 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>100000006518161100</t>
+          <t>100000003265158100</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>ранг 18: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 19: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24863,12 +24871,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>100000003265158100</t>
+          <t>100000008723830100</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>ранг 19: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 20: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24885,12 +24893,12 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>100000008723830100</t>
+          <t>100000002894076100</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>ранг 20: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 21: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24907,12 +24915,12 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>100000002894076100</t>
+          <t>100000004135268100</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>ранг 21: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 22: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24929,12 +24937,12 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>100000004135268100</t>
+          <t>100000003404627100</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>ранг 22: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 23: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24951,12 +24959,12 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>100000003404627100</t>
+          <t>100000005660203100</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>ранг 23: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 24: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24968,7 +24976,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -24978,7 +24986,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>ранг 24: в выгрузке есть даты, но нет времени</t>
+          <t>80% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -24990,17 +24998,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>100000005660203100</t>
+          <t>100000003071930100</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>80% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 25: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25012,7 +25020,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -25022,7 +25030,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>ранг 25: в выгрузке есть даты, но нет времени</t>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -25034,17 +25042,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>100000003071930100</t>
+          <t>100000001162560100</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 26: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25061,12 +25069,12 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>100000001162560100</t>
+          <t>100000004707703100</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>ранг 26: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 27: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25083,12 +25091,12 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>100000004707703100</t>
+          <t>100000007777377100</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>ранг 27: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 28: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25100,7 +25108,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -25110,7 +25118,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>ранг 28: в выгрузке есть даты, но нет времени</t>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -25122,17 +25130,17 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>100000007777377100</t>
+          <t>100000002781227100</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 29: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25149,39 +25157,17 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>100000002781227100</t>
+          <t>100000002443664100</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>ранг 29: в выгрузке есть даты, но нет времени</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>запрос</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>100000002443664100</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
           <t>ранг 30: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D45"/>
+  <autoFilter ref="A1:D44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(core): A6 clean export checkpoint [codex]
</commit_message>
<xml_diff>
--- a/out/evidence.xlsx
+++ b/out/evidence.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Транзакции-основания'!$A$1:$E$497</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Пути денег'!$A$1:$I$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Критерии'!$A$1:$E$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Границы данных'!$A$1:$D$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Границы данных'!$A$1:$D$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24253,10 +24253,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="47" customWidth="1" min="4" max="4"/>
@@ -24399,24 +24399,16 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>запрос</t>
+          <t>неполная выгрузка</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>100000008165763100</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>ранг 1: в выгрузке есть даты, но нет времени</t>
-        </is>
-      </c>
+          <t>audit.csv, run_meta.json</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -24431,12 +24423,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>100000003115284100</t>
+          <t>100000008165763100</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ранг 2: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 1: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24453,12 +24445,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>100000008686313100</t>
+          <t>100000003115284100</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>ранг 3: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 2: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24475,12 +24467,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>100000005339662100</t>
+          <t>100000008686313100</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>ранг 4: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 3: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24497,12 +24489,12 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>100000005527892100</t>
+          <t>100000005339662100</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>ранг 5: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 4: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24519,12 +24511,12 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>100000004299488100</t>
+          <t>100000005527892100</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>ранг 6: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 5: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24541,12 +24533,12 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>100000007055802100</t>
+          <t>100000004299488100</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>ранг 7: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 6: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24563,12 +24555,12 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>100000004070318100</t>
+          <t>100000007055802100</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>ранг 8: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 7: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24585,12 +24577,12 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>100000002398779100</t>
+          <t>100000004070318100</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>ранг 9: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 8: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24602,7 +24594,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -24612,7 +24604,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>67% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 9: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24624,17 +24616,17 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>100000008111003100</t>
+          <t>100000002398779100</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>ранг 10: в выгрузке есть даты, но нет времени</t>
+          <t>67% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -24651,12 +24643,12 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>100000008748408100</t>
+          <t>100000008111003100</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>ранг 11: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 10: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24673,12 +24665,12 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>100000004486525100</t>
+          <t>100000008748408100</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>ранг 12: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 11: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24695,12 +24687,12 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>100000004071080100</t>
+          <t>100000004486525100</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ранг 13: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 12: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24712,7 +24704,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -24722,7 +24714,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>60% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 13: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24734,17 +24726,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>100000003299365100</t>
+          <t>100000004071080100</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>ранг 14: в выгрузке есть даты, но нет времени</t>
+          <t>60% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -24761,12 +24753,12 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>100000004759121100</t>
+          <t>100000003299365100</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>ранг 15: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 14: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24783,12 +24775,12 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>100000003635170100</t>
+          <t>100000004759121100</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>ранг 16: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 15: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24805,12 +24797,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>100000001530983100</t>
+          <t>100000003635170100</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>ранг 17: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 16: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24827,12 +24819,12 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>100000006518161100</t>
+          <t>100000001530983100</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>ранг 18: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 17: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24849,12 +24841,12 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>100000003265158100</t>
+          <t>100000006518161100</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>ранг 19: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 18: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24871,12 +24863,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>100000008723830100</t>
+          <t>100000003265158100</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>ранг 20: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 19: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24893,12 +24885,12 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>100000002894076100</t>
+          <t>100000008723830100</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>ранг 21: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 20: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24915,12 +24907,12 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>100000004135268100</t>
+          <t>100000002894076100</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>ранг 22: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 21: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24937,12 +24929,12 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>100000003404627100</t>
+          <t>100000004135268100</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>ранг 23: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 22: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24959,12 +24951,12 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>100000005660203100</t>
+          <t>100000003404627100</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>ранг 24: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 23: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24976,7 +24968,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -24986,7 +24978,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>80% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 24: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24998,17 +24990,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>100000003071930100</t>
+          <t>100000005660203100</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>ранг 25: в выгрузке есть даты, но нет времени</t>
+          <t>80% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -25020,7 +25012,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -25030,7 +25022,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 25: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25042,17 +25034,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>100000001162560100</t>
+          <t>100000003071930100</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>ранг 26: в выгрузке есть даты, но нет времени</t>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -25069,12 +25061,12 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>100000004707703100</t>
+          <t>100000001162560100</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>ранг 27: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 26: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25091,12 +25083,12 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>100000007777377100</t>
+          <t>100000004707703100</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>ранг 28: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 27: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25108,7 +25100,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -25118,7 +25110,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 28: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25130,17 +25122,17 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>100000002781227100</t>
+          <t>100000007777377100</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>ранг 29: в выгрузке есть даты, но нет времени</t>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -25157,17 +25149,39 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
+          <t>100000002781227100</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>ранг 29: в выгрузке есть даты, но нет времени</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>запросить время транзакций для точного FlowTrace</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
           <t>100000002443664100</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>ранг 30: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D44"/>
+  <autoFilter ref="A1:D45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: clarify audit evidence and record compliance gaps [codex]
</commit_message>
<xml_diff>
--- a/out/evidence.xlsx
+++ b/out/evidence.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Транзакции-основания'!$A$1:$E$497</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Пути денег'!$A$1:$I$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Критерии'!$A$1:$E$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Границы данных'!$A$1:$D$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Границы данных'!$A$1:$D$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -520,7 +520,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -539,7 +539,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы: роль 0.30, деньги курьеров 0.28, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>кандидат в организаторы; связи вход/выход 15/17; деньги курьеров: модельно атрибутировано 150,166 ₸, seed с маршрутом 2; потеря seed-достижимости при удалении 0.46%; быстро отправлено 68%, пик плательщиков за день 4. Вклады в приоритет: роль 0.30, деньги курьеров 0.28, время 0.10; множитель 1.00. Контр: 87.1% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -562,7 +562,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr"/>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
@@ -581,7 +581,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: деньги курьеров 0.30, роль 0.24, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>признаки точки консолидации; связи вход/выход 8/2; деньги курьеров: модельно атрибутировано 815,000 ₸, seed с маршрутом 7; потеря seed-достижимости при удалении 0.28%; быстро отправлено 99%, пик плательщиков за день 7. Вклады в приоритет: деньги курьеров 0.30, роль 0.24, время 0.10; множитель 1.00. Контр: 62.3% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr"/>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -623,7 +623,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы: роль 0.30, деньги курьеров 0.24, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>кандидат в организаторы; связи вход/выход 6/7; деньги курьеров: модельно атрибутировано 225,181 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.09%; быстро отправлено 100%, пик плательщиков за день 2. Вклады в приоритет: роль 0.30, деньги курьеров 0.24, время 0.10; множитель 1.00. Контр: 88.2% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr"/>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="90" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
@@ -665,7 +665,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы: роль 0.30, деньги курьеров 0.22, оборот 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>кандидат в организаторы; связи вход/выход 4/4; деньги курьеров: модельно атрибутировано 39,925 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.18%; быстро отправлено 77%, пик плательщиков за день 2. Вклады в приоритет: роль 0.30, деньги курьеров 0.22, оборот 0.09; множитель 1.00. Контр: 80.3% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr"/>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
@@ -707,7 +707,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>кандидат в организаторы; связи вход/выход 3/8; деньги курьеров: модельно атрибутировано 70,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.23%; быстро отправлено 62%, пик плательщиков за день 1. Вклады в приоритет: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: 68.2% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr"/>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="90" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
@@ -749,7 +749,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: деньги курьеров 0.24, роль 0.24, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>признаки точки консолидации; связи вход/выход 6/2; деньги курьеров: модельно атрибутировано 575,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.09%; быстро отправлено 94%, пик плательщиков за день 3. Вклады в приоритет: деньги курьеров 0.24, роль 0.24, время 0.10; множитель 1.00. Контр: 67.1% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr"/>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -791,7 +791,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: деньги курьеров 0.24, роль 0.24, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>признаки точки консолидации; связи вход/выход 6/1; деньги курьеров: модельно атрибутировано 334,999 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.05%; быстро отправлено 100%, пик плательщиков за день 4. Вклады в приоритет: деньги курьеров 0.24, роль 0.24, время 0.10; множитель 1.00. Контр: 83.5% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr"/>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="90" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
@@ -833,7 +833,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>кандидат в организаторы; связи вход/выход 4/19; деньги курьеров: модельно атрибутировано 64,725 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.37%; быстро отправлено 54%, пик плательщиков за день 2. Вклады в приоритет: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: 68.8% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr"/>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
@@ -875,7 +875,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: роль 0.24, деньги курьеров 0.23, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>признаки точки консолидации; связи вход/выход 13/1; деньги курьеров: модельно атрибутировано 68,175 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.05%; быстро отправлено 100%, пик плательщиков за день 7. Вклады в приоритет: роль 0.24, деньги курьеров 0.23, время 0.10; множитель 1.00. Контр: 93.8% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr"/>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="90" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
@@ -917,7 +917,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: роль 0.24, деньги курьеров 0.23, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>признаки точки консолидации; связи вход/выход 6/1; деньги курьеров: модельно атрибутировано 86,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.18%; быстро отправлено 100%, пик плательщиков за день 2. Вклады в приоритет: роль 0.24, деньги курьеров 0.23, время 0.10; множитель 1.00. Контр: 61.4% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr"/>
     </row>
-    <row r="12" ht="45" customHeight="1">
+    <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
@@ -959,7 +959,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+          <t>признаки веерного распределения; связи вход/выход 1/21; деньги курьеров: модельно атрибутировано 360,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 1.25%; быстро отправлено 87%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -986,7 +986,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="90" customHeight="1">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: роль 0.24, деньги курьеров 0.21, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>признаки точки консолидации; связи вход/выход 8/2; деньги курьеров: модельно атрибутировано 17,900 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.05%; быстро отправлено 100%, пик плательщиков за день 5. Вклады в приоритет: роль 0.24, деньги курьеров 0.21, время 0.10; множитель 1.00. Контр: 95.0% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr"/>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: роль 0.24, деньги курьеров 0.23, время 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>признаки точки консолидации; связи вход/выход 9/2; деньги курьеров: модельно атрибутировано 73,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.09%; быстро отправлено 87%, пик плательщиков за день 2. Вклады в приоритет: роль 0.24, деньги курьеров 0.23, время 0.09; множитель 1.00. Контр: 69.4% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr"/>
     </row>
-    <row r="15" ht="45" customHeight="1">
+    <row r="15" ht="90" customHeight="1">
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.29, роль 0.15, время 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+          <t>признаки транзитного счёта; связи вход/выход 1/1; деньги курьеров: модельно атрибутировано 200,000 ₸, seed с маршрутом 4; потеря seed-достижимости при удалении 0.05%; быстро отправлено 100%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.29, роль 0.15, время 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1116,7 +1116,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
+    <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: роль 0.24, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>признаки точки консолидации; связи вход/выход 6/2; деньги курьеров: модельно атрибутировано 50,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.23%; быстро отправлено 52%, пик плательщиков за день 1. Вклады в приоритет: роль 0.24, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: 93.0% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr"/>
     </row>
-    <row r="17" ht="45" customHeight="1">
+    <row r="17" ht="90" customHeight="1">
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.27, роль 0.15, время 0.10; множитель 1.00. Контр: крупнейший плательщик дал 87% входящих (HHI 0.76).</t>
+          <t>признаки транзитного счёта; связи вход/выход 3/4; деньги курьеров: модельно атрибутировано 30,000 ₸, seed с маршрутом 5; потеря seed-достижимости при удалении 0.46%; быстро отправлено 100%, пик плательщиков за день 2. Вклады в приоритет: деньги курьеров 0.27, роль 0.15, время 0.10; множитель 1.00. Контр: крупнейший плательщик дал 87% входящих (HHI 0.76).</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1204,7 +1204,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения: деньги курьеров 0.28, роль 0.21, оборот 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>признаки веерного распределения; связи вход/выход 4/11; деньги курьеров: модельно атрибутировано 438,837 ₸, seed с маршрутом 2; потеря seed-достижимости при удалении 0.69%; быстро отправлено 16%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.28, роль 0.21, оборот 0.10; множитель 1.00. Контр: 22.2% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr"/>
     </row>
-    <row r="19" ht="45" customHeight="1">
+    <row r="19" ht="90" customHeight="1">
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.29, роль 0.15, оборот 0.09; множитель 1.00. Контр: крупнейший плательщик дал 88% входящих (HHI 0.78).</t>
+          <t>признаки транзитного счёта; связи вход/выход 3/2; деньги курьеров: модельно атрибутировано 544,200 ₸, seed с маршрутом 3; потеря seed-достижимости при удалении 0.18%; быстро отправлено 71%, пик плательщиков за день 2. Вклады в приоритет: деньги курьеров 0.29, роль 0.15, оборот 0.09; множитель 1.00. Контр: крупнейший плательщик дал 88% входящих (HHI 0.78).</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
+    <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.27, роль 0.15, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>признаки транзитного счёта; связи вход/выход 3/2; деньги курьеров: модельно атрибутировано 99,300 ₸, seed с маршрутом 2; потеря seed-достижимости при удалении 0.46%; быстро отправлено 100%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.27, роль 0.15, время 0.10; множитель 1.00. Контр: 32.0% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr"/>
     </row>
-    <row r="21" ht="45" customHeight="1">
+    <row r="21" ht="90" customHeight="1">
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
@@ -1353,7 +1353,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.24, роль 0.15, время 0.10; множитель 1.00. Контр: крупнейший плательщик дал 99% входящих (HHI 0.98).</t>
+          <t>признаки транзитного счёта; связи вход/выход 2/1; деньги курьеров: модельно атрибутировано 454,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.09%; быстро отправлено 100%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.15, время 0.10; множитель 1.00. Контр: крупнейший плательщик дал 99% входящих (HHI 0.98).</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1380,7 +1380,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
+    <row r="22" ht="105" customHeight="1">
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки: деньги курьеров 0.30, время 0.10, оборот 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>конечный получатель в пределах выгрузки; связи вход/выход 4/0; деньги курьеров: модельно атрибутировано 821,782 ₸, seed с маршрутом 4; компонент связности не учитывается: нет входящих или исходящих связей; быстро отправлено 0%, пик плательщиков за день 3. Вклады в приоритет: деньги курьеров 0.30, время 0.10, оборот 0.09; множитель 1.00. Контр: 26.8% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr"/>
     </row>
-    <row r="23" ht="45" customHeight="1">
+    <row r="23" ht="90" customHeight="1">
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.25, роль 0.15, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 86% входящих (HHI 0.76).</t>
+          <t>признаки транзитного счёта; связи вход/выход 2/3; деньги курьеров: модельно атрибутировано 1,064,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.14%; быстро отправлено 85%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.25, роль 0.15, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 86% входящих (HHI 0.76).</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1468,7 +1468,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="105" customHeight="1">
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки: деньги курьеров 0.30, время 0.10, оборот 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>конечный получатель в пределах выгрузки; связи вход/выход 4/0; деньги курьеров: модельно атрибутировано 465,000 ₸, seed с маршрутом 4; компонент связности не учитывается: нет входящих или исходящих связей; быстро отправлено 0%, пик плательщиков за день 3. Вклады в приоритет: деньги курьеров 0.30, время 0.10, оборот 0.09; множитель 1.00. Контр: 47.0% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr"/>
     </row>
-    <row r="25" ht="45" customHeight="1">
+    <row r="25" ht="90" customHeight="1">
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки: деньги курьеров 0.29, время 0.10, роль 0.09; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+          <t>конечный получатель в пределах выгрузки; связи вход/выход 1/2; деньги курьеров: модельно атрибутировано 402,899 ₸, seed с маршрутом 3; потеря seed-достижимости при удалении 0.09%; быстро отправлено 100%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.29, время 0.10, роль 0.09; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1556,7 +1556,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="30" customHeight="1">
+    <row r="26" ht="90" customHeight="1">
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки: деньги курьеров 0.29, время 0.10, роль 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
+          <t>конечный получатель в пределах выгрузки; связи вход/выход 3/1; деньги курьеров: модельно атрибутировано 227,610 ₸, seed с маршрутом 4; потеря seed-достижимости при удалении 0.14%; быстро отправлено 100%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.29, время 0.10, роль 0.09; множитель 1.00. Контр: 52.3% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr"/>
     </row>
-    <row r="27" ht="45" customHeight="1">
+    <row r="27" ht="90" customHeight="1">
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
@@ -1617,7 +1617,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+          <t>признаки веерного распределения; связи вход/выход 1/12; деньги курьеров: модельно атрибутировано 331,300 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.46%; быстро отправлено 15%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1644,7 +1644,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="45" customHeight="1">
+    <row r="28" ht="90" customHeight="1">
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
@@ -1663,7 +1663,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.24, роль 0.15, время 0.09; множитель 1.00. Контр: крупнейший плательщик дал 97% входящих (HHI 0.94).</t>
+          <t>признаки транзитного счёта; связи вход/выход 2/5; деньги курьеров: модельно атрибутировано 239,300 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.14%; быстро отправлено 89%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.15, время 0.09; множитель 1.00. Контр: крупнейший плательщик дал 97% входящих (HHI 0.94).</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1690,7 +1690,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="45" customHeight="1">
+    <row r="29" ht="90" customHeight="1">
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки: деньги курьеров 0.28, время 0.10, роль 0.09; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+          <t>конечный получатель в пределах выгрузки; связи вход/выход 1/2; деньги курьеров: модельно атрибутировано 306,290 ₸, seed с маршрутом 2; потеря seed-достижимости при удалении 0.28%; быстро отправлено 100%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.28, время 0.10, роль 0.09; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1736,7 +1736,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="45" customHeight="1">
+    <row r="30" ht="90" customHeight="1">
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.24, роль 0.15, оборот 0.08; множитель 1.00. Контр: крупнейший плательщик дал 76% входящих (HHI 0.63).</t>
+          <t>признаки транзитного счёта; связи вход/выход 2/3; деньги курьеров: модельно атрибутировано 191,168 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.09%; быстро отправлено 81%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.15, оборот 0.08; множитель 1.00. Контр: крупнейший плательщик дал 76% входящих (HHI 0.63).</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1782,7 +1782,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="45" customHeight="1">
+    <row r="31" ht="90" customHeight="1">
       <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки: деньги курьеров 0.27, время 0.10, роль 0.09; множитель 1.00. Контр: крупнейший плательщик дал 75% входящих (HHI 0.60).</t>
+          <t>конечный получатель в пределах выгрузки; связи вход/выход 3/0; деньги курьеров: модельно атрибутировано 74,880 ₸, seed с маршрутом 2; компонент связности не учитывается: нет входящих или исходящих связей; быстро отправлено 0%, пик плательщиков за день 3. Вклады в приоритет: деньги курьеров 0.27, время 0.10, роль 0.09; множитель 1.00. Контр: крупнейший плательщик дал 75% входящих (HHI 0.60).</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1885,7 +1885,7 @@
     <col width="15" customWidth="1" min="40" max="40"/>
     <col width="17" customWidth="1" min="41" max="41"/>
     <col width="15" customWidth="1" min="42" max="42"/>
-    <col width="66" customWidth="1" min="43" max="43"/>
+    <col width="63" customWidth="1" min="43" max="43"/>
     <col width="52" customWidth="1" min="44" max="44"/>
     <col width="14" customWidth="1" min="45" max="45"/>
     <col width="20" customWidth="1" min="46" max="46"/>
@@ -2165,7 +2165,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="90" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>100000001162560100</t>
@@ -2338,11 +2338,11 @@
       </c>
       <c r="BA2" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+          <t>признаки веерного распределения; связи вход/выход 1/12; деньги курьеров: модельно атрибутировано 331,300 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.46%; быстро отправлено 15%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>100000001530983100</t>
@@ -2511,11 +2511,11 @@
       </c>
       <c r="BA3" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения: деньги курьеров 0.28, роль 0.21, оборот 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>признаки веерного распределения; связи вход/выход 4/11; деньги курьеров: модельно атрибутировано 438,837 ₸, seed с маршрутом 2; потеря seed-достижимости при удалении 0.69%; быстро отправлено 16%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.28, роль 0.21, оборот 0.10; множитель 1.00. Контр: 22.2% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="90" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>100000002398779100</t>
@@ -2688,11 +2688,11 @@
       </c>
       <c r="BA4" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: роль 0.24, деньги курьеров 0.23, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="45" customHeight="1">
+          <t>признаки точки консолидации; связи вход/выход 13/1; деньги курьеров: модельно атрибутировано 68,175 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.05%; быстро отправлено 100%, пик плательщиков за день 7. Вклады в приоритет: роль 0.24, деньги курьеров 0.23, время 0.10; множитель 1.00. Контр: 93.8% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>100000002443664100</t>
@@ -2865,11 +2865,11 @@
       </c>
       <c r="BA5" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки: деньги курьеров 0.27, время 0.10, роль 0.09; множитель 1.00. Контр: крупнейший плательщик дал 75% входящих (HHI 0.60).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
+          <t>конечный получатель в пределах выгрузки; связи вход/выход 3/0; деньги курьеров: модельно атрибутировано 74,880 ₸, seed с маршрутом 2; компонент связности не учитывается: нет входящих или исходящих связей; быстро отправлено 0%, пик плательщиков за день 3. Вклады в приоритет: деньги курьеров 0.27, время 0.10, роль 0.09; множитель 1.00. Контр: крупнейший плательщик дал 75% входящих (HHI 0.60).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>100000002781227100</t>
@@ -3042,11 +3042,11 @@
       </c>
       <c r="BA6" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.24, роль 0.15, оборот 0.08; множитель 1.00. Контр: крупнейший плательщик дал 76% входящих (HHI 0.63).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+          <t>признаки транзитного счёта; связи вход/выход 2/3; деньги курьеров: модельно атрибутировано 191,168 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.09%; быстро отправлено 81%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.15, оборот 0.08; множитель 1.00. Контр: крупнейший плательщик дал 76% входящих (HHI 0.63).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="105" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>100000002894076100</t>
@@ -3215,11 +3215,11 @@
       </c>
       <c r="BA7" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки: деньги курьеров 0.30, время 0.10, оборот 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
+          <t>конечный получатель в пределах выгрузки; связи вход/выход 4/0; деньги курьеров: модельно атрибутировано 821,782 ₸, seed с маршрутом 4; компонент связности не учитывается: нет входящих или исходящих связей; быстро отправлено 0%, пик плательщиков за день 3. Вклады в приоритет: деньги курьеров 0.30, время 0.10, оборот 0.09; множитель 1.00. Контр: 26.8% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>100000003071930100</t>
@@ -3388,11 +3388,11 @@
       </c>
       <c r="BA8" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки: деньги курьеров 0.29, время 0.10, роль 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
+          <t>конечный получатель в пределах выгрузки; связи вход/выход 3/1; деньги курьеров: модельно атрибутировано 227,610 ₸, seed с маршрутом 4; потеря seed-достижимости при удалении 0.14%; быстро отправлено 100%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.29, время 0.10, роль 0.09; множитель 1.00. Контр: 52.3% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>100000003115284100</t>
@@ -3561,11 +3561,11 @@
       </c>
       <c r="BA9" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: деньги курьеров 0.30, роль 0.24, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
+          <t>признаки точки консолидации; связи вход/выход 8/2; деньги курьеров: модельно атрибутировано 815,000 ₸, seed с маршрутом 7; потеря seed-достижимости при удалении 0.28%; быстро отправлено 99%, пик плательщиков за день 7. Вклады в приоритет: деньги курьеров 0.30, роль 0.24, время 0.10; множитель 1.00. Контр: 62.3% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>100000003265158100</t>
@@ -3734,11 +3734,11 @@
       </c>
       <c r="BA10" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.27, роль 0.15, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
+          <t>признаки транзитного счёта; связи вход/выход 3/2; деньги курьеров: модельно атрибутировано 99,300 ₸, seed с маршрутом 2; потеря seed-достижимости при удалении 0.46%; быстро отправлено 100%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.27, роль 0.15, время 0.10; множитель 1.00. Контр: 32.0% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>100000003299365100</t>
@@ -3911,11 +3911,11 @@
       </c>
       <c r="BA11" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.29, роль 0.15, время 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
+          <t>признаки транзитного счёта; связи вход/выход 1/1; деньги курьеров: модельно атрибутировано 200,000 ₸, seed с маршрутом 4; потеря seed-достижимости при удалении 0.05%; быстро отправлено 100%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.29, роль 0.15, время 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="105" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>100000003404627100</t>
@@ -4084,11 +4084,11 @@
       </c>
       <c r="BA12" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки: деньги курьеров 0.30, время 0.10, оборот 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
+          <t>конечный получатель в пределах выгрузки; связи вход/выход 4/0; деньги курьеров: модельно атрибутировано 465,000 ₸, seed с маршрутом 4; компонент связности не учитывается: нет входящих или исходящих связей; быстро отправлено 0%, пик плательщиков за день 3. Вклады в приоритет: деньги курьеров 0.30, время 0.10, оборот 0.09; множитель 1.00. Контр: 47.0% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>100000003635170100</t>
@@ -4261,11 +4261,11 @@
       </c>
       <c r="BA13" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.27, роль 0.15, время 0.10; множитель 1.00. Контр: крупнейший плательщик дал 87% входящих (HHI 0.76).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
+          <t>признаки транзитного счёта; связи вход/выход 3/4; деньги курьеров: модельно атрибутировано 30,000 ₸, seed с маршрутом 5; потеря seed-достижимости при удалении 0.46%; быстро отправлено 100%, пик плательщиков за день 2. Вклады в приоритет: деньги курьеров 0.27, роль 0.15, время 0.10; множитель 1.00. Контр: крупнейший плательщик дал 87% входящих (HHI 0.76).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>100000004070318100</t>
@@ -4287,7 +4287,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы (0.95): входящих связей 4; исходящих связей 19. Контр: не выявлен</t>
+          <t>кандидат в организаторы (0.95): ключевых соседей 4→14 (порог 3/3); связей вход/выход 4/19. Контр: не выявлен</t>
         </is>
       </c>
       <c r="G14" s="4" t="n">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="AQ14" s="2" t="inlineStr">
         <is>
-          <t>входящих связей 4 | исходящих связей 19 | ключевых соседей 4→14</t>
+          <t>ключевых соседей 4→14 (порог 3/3) | связей вход/выход 4/19</t>
         </is>
       </c>
       <c r="AR14" s="2" t="inlineStr"/>
@@ -4438,11 +4438,11 @@
       </c>
       <c r="BA14" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+          <t>кандидат в организаторы; связи вход/выход 4/19; деньги курьеров: модельно атрибутировано 64,725 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.37%; быстро отправлено 54%, пик плательщиков за день 2. Вклады в приоритет: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: 68.8% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>100000004071080100</t>
@@ -4611,11 +4611,11 @@
       </c>
       <c r="BA15" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: роль 0.24, деньги курьеров 0.23, время 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1">
+          <t>признаки точки консолидации; связи вход/выход 9/2; деньги курьеров: модельно атрибутировано 73,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.09%; быстро отправлено 87%, пик плательщиков за день 2. Вклады в приоритет: роль 0.24, деньги курьеров 0.23, время 0.09; множитель 1.00. Контр: 69.4% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>100000004135268100</t>
@@ -4788,11 +4788,11 @@
       </c>
       <c r="BA16" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.25, роль 0.15, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 86% входящих (HHI 0.76).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
+          <t>признаки транзитного счёта; связи вход/выход 2/3; деньги курьеров: модельно атрибутировано 1,064,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.14%; быстро отправлено 85%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.25, роль 0.15, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 86% входящих (HHI 0.76).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>100000004299488100</t>
@@ -4961,11 +4961,11 @@
       </c>
       <c r="BA17" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: деньги курьеров 0.24, роль 0.24, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
+          <t>признаки точки консолидации; связи вход/выход 6/2; деньги курьеров: модельно атрибутировано 575,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.09%; быстро отправлено 94%, пик плательщиков за день 3. Вклады в приоритет: деньги курьеров 0.24, роль 0.24, время 0.10; множитель 1.00. Контр: 67.1% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>100000004486525100</t>
@@ -5134,11 +5134,11 @@
       </c>
       <c r="BA18" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: роль 0.24, деньги курьеров 0.21, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="45" customHeight="1">
+          <t>признаки точки консолидации; связи вход/выход 8/2; деньги курьеров: модельно атрибутировано 17,900 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.05%; быстро отправлено 100%, пик плательщиков за день 5. Вклады в приоритет: роль 0.24, деньги курьеров 0.21, время 0.10; множитель 1.00. Контр: 95.0% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>100000004707703100</t>
@@ -5311,11 +5311,11 @@
       </c>
       <c r="BA19" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.24, роль 0.15, время 0.09; множитель 1.00. Контр: крупнейший плательщик дал 97% входящих (HHI 0.94).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
+          <t>признаки транзитного счёта; связи вход/выход 2/5; деньги курьеров: модельно атрибутировано 239,300 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.14%; быстро отправлено 89%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.15, время 0.09; множитель 1.00. Контр: крупнейший плательщик дал 97% входящих (HHI 0.94).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>100000004759121100</t>
@@ -5484,11 +5484,11 @@
       </c>
       <c r="BA20" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: роль 0.24, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
+          <t>признаки точки консолидации; связи вход/выход 6/2; деньги курьеров: модельно атрибутировано 50,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.23%; быстро отправлено 52%, пик плательщиков за день 1. Вклады в приоритет: роль 0.24, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: 93.0% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>100000005339662100</t>
@@ -5510,7 +5510,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы (0.65): входящих связей 4; исходящих связей 4. Контр: не выявлен</t>
+          <t>кандидат в организаторы (0.65): ключевых соседей 3→3 (порог 3/3); связей вход/выход 4/4. Контр: не выявлен</t>
         </is>
       </c>
       <c r="G21" s="4" t="n">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="AQ21" s="2" t="inlineStr">
         <is>
-          <t>входящих связей 4 | исходящих связей 4 | ключевых соседей 3→3</t>
+          <t>ключевых соседей 3→3 (порог 3/3) | связей вход/выход 4/4</t>
         </is>
       </c>
       <c r="AR21" s="2" t="inlineStr"/>
@@ -5657,11 +5657,11 @@
       </c>
       <c r="BA21" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы: роль 0.30, деньги курьеров 0.22, оборот 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
+          <t>кандидат в организаторы; связи вход/выход 4/4; деньги курьеров: модельно атрибутировано 39,925 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.18%; быстро отправлено 77%, пик плательщиков за день 2. Вклады в приоритет: роль 0.30, деньги курьеров 0.22, оборот 0.09; множитель 1.00. Контр: 80.3% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="90" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>100000005527892100</t>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы (0.65): входящих связей 3; исходящих связей 8. Контр: не выявлен</t>
+          <t>кандидат в организаторы (0.65): ключевых соседей 3→3 (порог 3/3); связей вход/выход 3/8. Контр: не выявлен</t>
         </is>
       </c>
       <c r="G22" s="4" t="n">
@@ -5800,7 +5800,7 @@
       </c>
       <c r="AQ22" s="2" t="inlineStr">
         <is>
-          <t>входящих связей 3 | исходящих связей 8 | ключевых соседей 3→3</t>
+          <t>ключевых соседей 3→3 (порог 3/3) | связей вход/выход 3/8</t>
         </is>
       </c>
       <c r="AR22" s="2" t="inlineStr"/>
@@ -5830,11 +5830,11 @@
       </c>
       <c r="BA22" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="45" customHeight="1">
+          <t>кандидат в организаторы; связи вход/выход 3/8; деньги курьеров: модельно атрибутировано 70,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.23%; быстро отправлено 62%, пик плательщиков за день 1. Вклады в приоритет: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: 68.2% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="90" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>100000005660203100</t>
@@ -6007,11 +6007,11 @@
       </c>
       <c r="BA23" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки: деньги курьеров 0.29, время 0.10, роль 0.09; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="45" customHeight="1">
+          <t>конечный получатель в пределах выгрузки; связи вход/выход 1/2; деньги курьеров: модельно атрибутировано 402,899 ₸, seed с маршрутом 3; потеря seed-достижимости при удалении 0.09%; быстро отправлено 100%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.29, время 0.10, роль 0.09; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="90" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
           <t>100000006518161100</t>
@@ -6184,11 +6184,11 @@
       </c>
       <c r="BA24" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.29, роль 0.15, оборот 0.09; множитель 1.00. Контр: крупнейший плательщик дал 88% входящих (HHI 0.78).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
+          <t>признаки транзитного счёта; связи вход/выход 3/2; деньги курьеров: модельно атрибутировано 544,200 ₸, seed с маршрутом 3; потеря seed-достижимости при удалении 0.18%; быстро отправлено 71%, пик плательщиков за день 2. Вклады в приоритет: деньги курьеров 0.29, роль 0.15, оборот 0.09; множитель 1.00. Контр: крупнейший плательщик дал 88% входящих (HHI 0.78).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="90" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t>100000007055802100</t>
@@ -6357,11 +6357,11 @@
       </c>
       <c r="BA25" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: деньги курьеров 0.24, роль 0.24, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="45" customHeight="1">
+          <t>признаки точки консолидации; связи вход/выход 6/1; деньги курьеров: модельно атрибутировано 334,999 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.05%; быстро отправлено 100%, пик плательщиков за день 4. Вклады в приоритет: деньги курьеров 0.24, роль 0.24, время 0.10; множитель 1.00. Контр: 83.5% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="90" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t>100000007777377100</t>
@@ -6534,11 +6534,11 @@
       </c>
       <c r="BA26" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки: деньги курьеров 0.28, время 0.10, роль 0.09; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
+          <t>конечный получатель в пределах выгрузки; связи вход/выход 1/2; деньги курьеров: модельно атрибутировано 306,290 ₸, seed с маршрутом 2; потеря seed-достижимости при удалении 0.28%; быстро отправлено 100%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.28, время 0.10, роль 0.09; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="90" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>100000008111003100</t>
@@ -6707,11 +6707,11 @@
       </c>
       <c r="BA27" s="2" t="inlineStr">
         <is>
-          <t>признаки точки консолидации: роль 0.24, деньги курьеров 0.23, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
+          <t>признаки точки консолидации; связи вход/выход 6/1; деньги курьеров: модельно атрибутировано 86,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.18%; быстро отправлено 100%, пик плательщиков за день 2. Вклады в приоритет: роль 0.24, деньги курьеров 0.23, время 0.10; множитель 1.00. Контр: 61.4% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t>100000008165763100</t>
@@ -6733,7 +6733,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы (0.80): входящих связей 15; исходящих связей 17. Контр: не выявлен</t>
+          <t>кандидат в организаторы (0.80): связей вход/выход 15/17 (порог 5/10); ключевых соседей 10→2. Контр: не выявлен</t>
         </is>
       </c>
       <c r="G28" s="4" t="n">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="AQ28" s="2" t="inlineStr">
         <is>
-          <t>входящих связей 15 | исходящих связей 17 | ключевых соседей 10→2</t>
+          <t>связей вход/выход 15/17 (порог 5/10) | ключевых соседей 10→2</t>
         </is>
       </c>
       <c r="AR28" s="2" t="inlineStr"/>
@@ -6884,11 +6884,11 @@
       </c>
       <c r="BA28" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы: роль 0.30, деньги курьеров 0.28, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
+          <t>кандидат в организаторы; связи вход/выход 15/17; деньги курьеров: модельно атрибутировано 150,166 ₸, seed с маршрутом 2; потеря seed-достижимости при удалении 0.46%; быстро отправлено 68%, пик плательщиков за день 4. Вклады в приоритет: роль 0.30, деньги курьеров 0.28, время 0.10; множитель 1.00. Контр: 87.1% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="90" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>100000008686313100</t>
@@ -6910,7 +6910,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы (0.75): входящих связей 6; исходящих связей 7. Контр: не выявлен</t>
+          <t>кандидат в организаторы (0.75): ключевых соседей 5→5 (порог 3/3); связей вход/выход 6/7. Контр: не выявлен</t>
         </is>
       </c>
       <c r="G29" s="4" t="n">
@@ -7031,7 +7031,7 @@
       </c>
       <c r="AQ29" s="2" t="inlineStr">
         <is>
-          <t>входящих связей 6 | исходящих связей 7 | ключевых соседей 5→5</t>
+          <t>ключевых соседей 5→5 (порог 3/3) | связей вход/выход 6/7</t>
         </is>
       </c>
       <c r="AR29" s="2" t="inlineStr"/>
@@ -7061,11 +7061,11 @@
       </c>
       <c r="BA29" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы: роль 0.30, деньги курьеров 0.24, время 0.10; множитель 1.00. Контр: только даты и 4 колена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="45" customHeight="1">
+          <t>кандидат в организаторы; связи вход/выход 6/7; деньги курьеров: модельно атрибутировано 225,181 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.09%; быстро отправлено 100%, пик плательщиков за день 2. Вклады в приоритет: роль 0.30, деньги курьеров 0.24, время 0.10; множитель 1.00. Контр: 88.2% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="90" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t>100000008723830100</t>
@@ -7238,11 +7238,11 @@
       </c>
       <c r="BA30" s="2" t="inlineStr">
         <is>
-          <t>признаки транзитного счёта: деньги курьеров 0.24, роль 0.15, время 0.10; множитель 1.00. Контр: крупнейший плательщик дал 99% входящих (HHI 0.98).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="45" customHeight="1">
+          <t>признаки транзитного счёта; связи вход/выход 2/1; деньги курьеров: модельно атрибутировано 454,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.09%; быстро отправлено 100%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.15, время 0.10; множитель 1.00. Контр: крупнейший плательщик дал 99% входящих (HHI 0.98).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="90" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>100000008748408100</t>
@@ -7415,7 +7415,7 @@
       </c>
       <c r="BA31" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+          <t>признаки веерного распределения; связи вход/выход 1/21; деньги курьеров: модельно атрибутировано 360,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 1.25%; быстро отправлено 87%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
         </is>
       </c>
     </row>
@@ -24253,10 +24253,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="47" customWidth="1" min="4" max="4"/>
@@ -24399,16 +24399,24 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>неполная выгрузка</t>
+          <t>запрос</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>audit.csv, run_meta.json</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
+          <t>запросить время транзакций для точного FlowTrace</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>100000008165763100</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>ранг 1: в выгрузке есть даты, но нет времени</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -24423,12 +24431,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>100000008165763100</t>
+          <t>100000003115284100</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ранг 1: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 2: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24445,12 +24453,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>100000003115284100</t>
+          <t>100000008686313100</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>ранг 2: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 3: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24467,12 +24475,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>100000008686313100</t>
+          <t>100000005339662100</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>ранг 3: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 4: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24489,12 +24497,12 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>100000005339662100</t>
+          <t>100000005527892100</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>ранг 4: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 5: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24511,12 +24519,12 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>100000005527892100</t>
+          <t>100000004299488100</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>ранг 5: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 6: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24533,12 +24541,12 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>100000004299488100</t>
+          <t>100000007055802100</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>ранг 6: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 7: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24555,12 +24563,12 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>100000007055802100</t>
+          <t>100000004070318100</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>ранг 7: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 8: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24577,12 +24585,12 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>100000004070318100</t>
+          <t>100000002398779100</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>ранг 8: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 9: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24594,7 +24602,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -24604,7 +24612,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>ранг 9: в выгрузке есть даты, но нет времени</t>
+          <t>67% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -24616,17 +24624,17 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>100000002398779100</t>
+          <t>100000008111003100</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>67% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 10: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24643,12 +24651,12 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>100000008111003100</t>
+          <t>100000008748408100</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>ранг 10: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 11: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24665,12 +24673,12 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>100000008748408100</t>
+          <t>100000004486525100</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>ранг 11: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 12: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24687,12 +24695,12 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>100000004486525100</t>
+          <t>100000004071080100</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ранг 12: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 13: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24704,7 +24712,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -24714,7 +24722,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>ранг 13: в выгрузке есть даты, но нет времени</t>
+          <t>60% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -24726,17 +24734,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>100000004071080100</t>
+          <t>100000003299365100</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>60% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 14: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24753,12 +24761,12 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>100000003299365100</t>
+          <t>100000004759121100</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>ранг 14: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 15: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24775,12 +24783,12 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>100000004759121100</t>
+          <t>100000003635170100</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>ранг 15: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 16: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24797,12 +24805,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>100000003635170100</t>
+          <t>100000001530983100</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>ранг 16: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 17: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24819,12 +24827,12 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>100000001530983100</t>
+          <t>100000006518161100</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>ранг 17: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 18: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24841,12 +24849,12 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>100000006518161100</t>
+          <t>100000003265158100</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>ранг 18: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 19: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24863,12 +24871,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>100000003265158100</t>
+          <t>100000008723830100</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>ранг 19: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 20: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24885,12 +24893,12 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>100000008723830100</t>
+          <t>100000002894076100</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>ранг 20: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 21: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24907,12 +24915,12 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>100000002894076100</t>
+          <t>100000004135268100</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>ранг 21: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 22: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24929,12 +24937,12 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>100000004135268100</t>
+          <t>100000003404627100</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>ранг 22: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 23: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24951,12 +24959,12 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>100000003404627100</t>
+          <t>100000005660203100</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>ранг 23: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 24: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -24968,7 +24976,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -24978,7 +24986,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>ранг 24: в выгрузке есть даты, но нет времени</t>
+          <t>80% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -24990,17 +24998,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>100000005660203100</t>
+          <t>100000003071930100</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>80% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 25: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25012,7 +25020,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -25022,7 +25030,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>ранг 25: в выгрузке есть даты, но нет времени</t>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -25034,17 +25042,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>100000003071930100</t>
+          <t>100000001162560100</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 26: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25061,12 +25069,12 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>100000001162560100</t>
+          <t>100000004707703100</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>ранг 26: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 27: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25083,12 +25091,12 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>100000004707703100</t>
+          <t>100000007777377100</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>ранг 27: в выгрузке есть даты, но нет времени</t>
+          <t>ранг 28: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25100,7 +25108,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
+          <t>запросить переводы &lt; 5 000 ₸</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -25110,7 +25118,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>ранг 28: в выгрузке есть даты, но нет времени</t>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
         </is>
       </c>
     </row>
@@ -25122,17 +25130,17 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>запросить переводы &lt; 5 000 ₸</t>
+          <t>запросить время транзакций для точного FlowTrace</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>100000007777377100</t>
+          <t>100000002781227100</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+          <t>ранг 29: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
@@ -25149,39 +25157,17 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>100000002781227100</t>
+          <t>100000002443664100</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>ранг 29: в выгрузке есть даты, но нет времени</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>запрос</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>запросить время транзакций для точного FlowTrace</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>100000002443664100</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
           <t>ранг 30: в выгрузке есть даты, но нет времени</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D45"/>
+  <autoFilter ref="A1:D44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: complete audit and analyst workflow [codex]
</commit_message>
<xml_diff>
--- a/out/evidence.xlsx
+++ b/out/evidence.xlsx
@@ -19,8 +19,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Признаки'!$A$1:$BA$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Транзакции-основания'!$A$1:$E$497</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Пути денег'!$A$1:$I$121</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Критерии'!$A$1:$E$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Границы данных'!$A$1:$D$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Критерии'!$A$1:$E$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Границы данных'!$A$1:$D$219</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,7 +465,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -707,7 +707,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы; связи вход/выход 3/8; деньги курьеров: модельно атрибутировано 70,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.23%; быстро отправлено 62%, пик плательщиков за день 1. Вклады в приоритет: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: 68.2% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+          <t>кандидат в организаторы; связи вход/выход 3/8; деньги курьеров: модельно атрибутировано 70,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.23%; быстро отправлено 62%, пик плательщиков за день 1. Вклады в приоритет: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: исходящие превышают наблюдаемые входящие ×2.5; возможен начальный остаток или средства вне выборки.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -728,7 +728,11 @@
       <c r="I6" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>исходящие превышают наблюдаемые входящие ×2.5; возможен начальный остаток или средства вне выборки</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -833,7 +837,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы; связи вход/выход 4/19; деньги курьеров: модельно атрибутировано 64,725 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.37%; быстро отправлено 54%, пик плательщиков за день 2. Вклады в приоритет: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: 68.8% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+          <t>кандидат в организаторы; связи вход/выход 4/19; деньги курьеров: модельно атрибутировано 64,725 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.37%; быстро отправлено 54%, пик плательщиков за день 2. Вклады в приоритет: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: исходящие превышают наблюдаемые входящие ×2.7; возможен начальный остаток или средства вне выборки.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -854,7 +858,11 @@
       <c r="I9" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>исходящие превышают наблюдаемые входящие ×2.7; возможен начальный остаток или средства вне выборки</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -959,7 +967,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения; связи вход/выход 1/21; деньги курьеров: модельно атрибутировано 360,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 1.25%; быстро отправлено 87%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+          <t>признаки веерного распределения; связи вход/выход 1/21; деньги курьеров: модельно атрибутировано 360,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 1.25%; быстро отправлено 87%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: исходящие превышают наблюдаемые входящие ×4.2; возможен начальный остаток или средства вне выборки.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -982,7 +990,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>крупнейший плательщик дал 100% входящих (HHI 1.00)</t>
+          <t>исходящие превышают наблюдаемые входящие ×4.2; возможен начальный остаток или средства вне выборки | крупнейший плательщик дал 100% входящих (HHI 1.00)</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1231,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения; связи вход/выход 4/11; деньги курьеров: модельно атрибутировано 438,837 ₸, seed с маршрутом 2; потеря seed-достижимости при удалении 0.69%; быстро отправлено 16%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.28, роль 0.21, оборот 0.10; множитель 1.00. Контр: 22.2% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+          <t>признаки веерного распределения; связи вход/выход 4/11; деньги курьеров: модельно атрибутировано 438,837 ₸, seed с маршрутом 2; потеря seed-достижимости при удалении 0.69%; быстро отправлено 16%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.28, роль 0.21, оборот 0.10; множитель 1.00. Контр: исходящие превышают наблюдаемые входящие ×3.2; возможен начальный остаток или средства вне выборки.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1244,7 +1252,11 @@
       <c r="I18" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>исходящие превышают наблюдаемые входящие ×3.2; возможен начальный остаток или средства вне выборки</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="2" t="n">
@@ -1617,7 +1629,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения; связи вход/выход 1/12; деньги курьеров: модельно атрибутировано 331,300 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.46%; быстро отправлено 15%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+          <t>признаки веерного распределения; связи вход/выход 1/12; деньги курьеров: модельно атрибутировано 331,300 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.46%; быстро отправлено 15%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: исходящие превышают наблюдаемые входящие ×8.8; возможен начальный остаток или средства вне выборки.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1640,7 +1652,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>крупнейший плательщик дал 100% входящих (HHI 1.00)</t>
+          <t>исходящие превышают наблюдаемые входящие ×8.8; возможен начальный остаток или средства вне выборки | крупнейший плательщик дал 100% входящих (HHI 1.00)</t>
         </is>
       </c>
     </row>
@@ -1885,8 +1897,8 @@
     <col width="15" customWidth="1" min="40" max="40"/>
     <col width="17" customWidth="1" min="41" max="41"/>
     <col width="15" customWidth="1" min="42" max="42"/>
-    <col width="63" customWidth="1" min="43" max="43"/>
-    <col width="52" customWidth="1" min="44" max="44"/>
+    <col width="70" customWidth="1" min="43" max="43"/>
+    <col width="70" customWidth="1" min="44" max="44"/>
     <col width="14" customWidth="1" min="45" max="45"/>
     <col width="20" customWidth="1" min="46" max="46"/>
     <col width="20" customWidth="1" min="47" max="47"/>
@@ -2187,7 +2199,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения (0.44): получателей 12; отправлено 2.9 млн ₸. Контр: 1 плательщик 100%</t>
+          <t>признаки веерного распределения (0.44): получателей 12; отправлено 2.9 млн ₸. Контр: исходящие/входящие ×8.8; баланс неполон</t>
         </is>
       </c>
       <c r="G2" s="4" t="n">
@@ -2309,7 +2321,7 @@
       </c>
       <c r="AR2" s="2" t="inlineStr">
         <is>
-          <t>крупнейший плательщик дал 100% входящих (HHI 1.00)</t>
+          <t>исходящие превышают наблюдаемые входящие ×8.8; возможен начальный остаток или средства вне выборки | крупнейший плательщик дал 100% входящих (HHI 1.00)</t>
         </is>
       </c>
       <c r="AS2" s="4" t="n">
@@ -2338,7 +2350,7 @@
       </c>
       <c r="BA2" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения; связи вход/выход 1/12; деньги курьеров: модельно атрибутировано 331,300 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.46%; быстро отправлено 15%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+          <t>признаки веерного распределения; связи вход/выход 1/12; деньги курьеров: модельно атрибутировано 331,300 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.46%; быстро отправлено 15%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: исходящие превышают наблюдаемые входящие ×8.8; возможен начальный остаток или средства вне выборки.</t>
         </is>
       </c>
     </row>
@@ -2364,7 +2376,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения (0.41): получателей 11; отправлено 1.8 млн ₸. Контр: не выявлен</t>
+          <t>признаки веерного распределения (0.41): получателей 11; отправлено 1.8 млн ₸. Контр: исходящие/входящие ×3.2; баланс неполон</t>
         </is>
       </c>
       <c r="G3" s="4" t="n">
@@ -2484,7 +2496,11 @@
           <t>получателей 11 | отправлено 1.8 млн ₸ | быстро отправлено 16%</t>
         </is>
       </c>
-      <c r="AR3" s="2" t="inlineStr"/>
+      <c r="AR3" s="2" t="inlineStr">
+        <is>
+          <t>исходящие превышают наблюдаемые входящие ×3.2; возможен начальный остаток или средства вне выборки</t>
+        </is>
+      </c>
       <c r="AS3" s="4" t="n">
         <v>0.7</v>
       </c>
@@ -2511,7 +2527,7 @@
       </c>
       <c r="BA3" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения; связи вход/выход 4/11; деньги курьеров: модельно атрибутировано 438,837 ₸, seed с маршрутом 2; потеря seed-достижимости при удалении 0.69%; быстро отправлено 16%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.28, роль 0.21, оборот 0.10; множитель 1.00. Контр: 22.2% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+          <t>признаки веерного распределения; связи вход/выход 4/11; деньги курьеров: модельно атрибутировано 438,837 ₸, seed с маршрутом 2; потеря seed-достижимости при удалении 0.69%; быстро отправлено 16%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.28, роль 0.21, оборот 0.10; множитель 1.00. Контр: исходящие превышают наблюдаемые входящие ×3.2; возможен начальный остаток или средства вне выборки.</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3257,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки (0.84): колено 1; исходящих связей 1. Контр: не выявлен</t>
+          <t>конечный получатель в пределах выгрузки (0.84): исходящие 1.05% входящих (порог &lt;10%); колено 1, исходящих связей 1. Контр: не выявлен</t>
         </is>
       </c>
       <c r="G8" s="4" t="n">
@@ -3358,7 +3374,7 @@
       </c>
       <c r="AQ8" s="2" t="inlineStr">
         <is>
-          <t>колено 1 | исходящих связей 1 | прослежено 48% входящих</t>
+          <t>исходящие 1.05% входящих (порог &lt;10%) | колено 1, исходящих связей 1 | прослежено 48% входящих</t>
         </is>
       </c>
       <c r="AR8" s="2" t="inlineStr"/>
@@ -4287,7 +4303,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы (0.95): ключевых соседей 4→14 (порог 3/3); связей вход/выход 4/19. Контр: не выявлен</t>
+          <t>кандидат в организаторы (0.95): ключевых соседей 4→14 (порог 3/3); связей вход/выход 4/19. Контр: исходящие/входящие ×2.7; баланс неполон</t>
         </is>
       </c>
       <c r="G14" s="4" t="n">
@@ -4411,7 +4427,11 @@
           <t>ключевых соседей 4→14 (порог 3/3) | связей вход/выход 4/19</t>
         </is>
       </c>
-      <c r="AR14" s="2" t="inlineStr"/>
+      <c r="AR14" s="2" t="inlineStr">
+        <is>
+          <t>исходящие превышают наблюдаемые входящие ×2.7; возможен начальный остаток или средства вне выборки</t>
+        </is>
+      </c>
       <c r="AS14" s="4" t="n">
         <v>1</v>
       </c>
@@ -4438,7 +4458,7 @@
       </c>
       <c r="BA14" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы; связи вход/выход 4/19; деньги курьеров: модельно атрибутировано 64,725 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.37%; быстро отправлено 54%, пик плательщиков за день 2. Вклады в приоритет: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: 68.8% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+          <t>кандидат в организаторы; связи вход/выход 4/19; деньги курьеров: модельно атрибутировано 64,725 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.37%; быстро отправлено 54%, пик плательщиков за день 2. Вклады в приоритет: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: исходящие превышают наблюдаемые входящие ×2.7; возможен начальный остаток или средства вне выборки.</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5703,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы (0.65): ключевых соседей 3→3 (порог 3/3); связей вход/выход 3/8. Контр: не выявлен</t>
+          <t>кандидат в организаторы (0.65): ключевых соседей 3→3 (порог 3/3); связей вход/выход 3/8. Контр: исходящие/входящие ×2.5; баланс неполон</t>
         </is>
       </c>
       <c r="G22" s="4" t="n">
@@ -5803,7 +5823,11 @@
           <t>ключевых соседей 3→3 (порог 3/3) | связей вход/выход 3/8</t>
         </is>
       </c>
-      <c r="AR22" s="2" t="inlineStr"/>
+      <c r="AR22" s="2" t="inlineStr">
+        <is>
+          <t>исходящие превышают наблюдаемые входящие ×2.5; возможен начальный остаток или средства вне выборки</t>
+        </is>
+      </c>
       <c r="AS22" s="4" t="n">
         <v>1</v>
       </c>
@@ -5830,7 +5854,7 @@
       </c>
       <c r="BA22" s="2" t="inlineStr">
         <is>
-          <t>кандидат в организаторы; связи вход/выход 3/8; деньги курьеров: модельно атрибутировано 70,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.23%; быстро отправлено 62%, пик плательщиков за день 1. Вклады в приоритет: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: 68.2% входящих не атрибутировано seed; маршрут по датам не доказывает происхождение средств.</t>
+          <t>кандидат в организаторы; связи вход/выход 3/8; деньги курьеров: модельно атрибутировано 70,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 0.23%; быстро отправлено 62%, пик плательщиков за день 1. Вклады в приоритет: роль 0.30, деньги курьеров 0.23, оборот 0.09; множитель 1.00. Контр: исходящие превышают наблюдаемые входящие ×2.5; возможен начальный остаток или средства вне выборки.</t>
         </is>
       </c>
     </row>
@@ -5856,7 +5880,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки (0.91): колено 2; исходящих связей 2. Контр: 1 плательщик 100%</t>
+          <t>конечный получатель в пределах выгрузки (0.91): исходящие 7.16% входящих (порог &lt;10%); колено 2, исходящих связей 2. Контр: 1 плательщик 100%</t>
         </is>
       </c>
       <c r="G23" s="4" t="n">
@@ -5973,7 +5997,7 @@
       </c>
       <c r="AQ23" s="2" t="inlineStr">
         <is>
-          <t>колено 2 | исходящих связей 2 | прослежено 70% входящих</t>
+          <t>исходящие 7.16% входящих (порог &lt;10%) | колено 2, исходящих связей 2 | прослежено 70% входящих</t>
         </is>
       </c>
       <c r="AR23" s="2" t="inlineStr">
@@ -6383,7 +6407,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>конечный получатель в пределах выгрузки (0.90): колено 2; исходящих связей 2. Контр: 1 плательщик 100%</t>
+          <t>конечный получатель в пределах выгрузки (0.90): исходящие 2.19% входящих (порог &lt;10%); колено 2, исходящих связей 2. Контр: 1 плательщик 100%</t>
         </is>
       </c>
       <c r="G26" s="4" t="n">
@@ -6500,7 +6524,7 @@
       </c>
       <c r="AQ26" s="2" t="inlineStr">
         <is>
-          <t>колено 2 | исходящих связей 2 | прослежено 67% входящих</t>
+          <t>исходящие 2.19% входящих (порог &lt;10%) | колено 2, исходящих связей 2 | прослежено 67% входящих</t>
         </is>
       </c>
       <c r="AR26" s="2" t="inlineStr">
@@ -7264,7 +7288,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения (0.72): получателей 21; отправлено 1.5 млн ₸. Контр: 1 плательщик 100%</t>
+          <t>признаки веерного распределения (0.72): получателей 21; отправлено 1.5 млн ₸. Контр: исходящие/входящие ×4.2; баланс неполон</t>
         </is>
       </c>
       <c r="G31" s="4" t="n">
@@ -7386,7 +7410,7 @@
       </c>
       <c r="AR31" s="2" t="inlineStr">
         <is>
-          <t>крупнейший плательщик дал 100% входящих (HHI 1.00)</t>
+          <t>исходящие превышают наблюдаемые входящие ×4.2; возможен начальный остаток или средства вне выборки | крупнейший плательщик дал 100% входящих (HHI 1.00)</t>
         </is>
       </c>
       <c r="AS31" s="4" t="n">
@@ -7415,7 +7439,7 @@
       </c>
       <c r="BA31" s="2" t="inlineStr">
         <is>
-          <t>признаки веерного распределения; связи вход/выход 1/21; деньги курьеров: модельно атрибутировано 360,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 1.25%; быстро отправлено 87%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: крупнейший плательщик дал 100% входящих (HHI 1.00).</t>
+          <t>признаки веерного распределения; связи вход/выход 1/21; деньги курьеров: модельно атрибутировано 360,000 ₸, seed с маршрутом 1; потеря seed-достижимости при удалении 1.25%; быстро отправлено 87%, пик плательщиков за день 1. Вклады в приоритет: деньги курьеров 0.24, роль 0.21, оборот 0.10; множитель 1.00. Контр: исходящие превышают наблюдаемые входящие ×4.2; возможен начальный остаток или средства вне выборки.</t>
         </is>
       </c>
     </row>
@@ -7431,7 +7455,7 @@
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>[{"параметр": "AGG_MAX_HHI", "значение": "0.15"}, {"параметр": "AGG_MIN_ACTIVE_DAYS", "значение": "12"}, {"параметр": "AGG_MIN_IN_DEG", "значение": "10"}, {"параметр": "AGG_MIN_ONE_OFF", "значение": "0.8"}, {"параметр": "AMBIGUOUS_MARGIN", "значение": "0.1"}, {"параметр": "CHRONO_GAPS", "значение": "{\"any\": 31, \"7d\": 7, \"2d\": 2}"}, {"параметр": "CONF_LEVELS", "значение": "[0.5, 0.75]"}, {"параметр": "CONS_MIN_IN_DEG", "значение": "5"}, {"параметр": "COORD_MIN_KEY_LINKS", "значение": "3"}, {"параметр": "DIST_MIN_OUT_DEG", "значение": "10"}, {"параметр": "EXT_FUNDING_MAX_TRACKED_OUT", "значение": "0.1"}, {"параметр": "EXT_FUNDING_PT", "значение": "2.0"}, {"параметр": "FAST_DAYS", "значение": "2"}, {"параметр": "HHI_DOMINANT", "значение": "0.5"}, {"параметр": "MULT", "значение": "{\"no_chrono\": 0.5, \"external_funding\": 0.7, \"seed\": 0.6, \"seed_above_bottom\": 0.8, \"payer\": 0.2, \"excluded\": 0.0}"}, {"параметр": "NEAR_THRESHOLD", "значение": "[5000, 7000]"}, {"параметр": "PATH_GAP_DAYS", "значение": "7"}, {"параметр": "PAYER_MAX_KZT", "значение": "100000"}, {"параметр": "PAYER_MAX_OUT_DEG", "значение": "2"}, {"параметр": "PAYER_MAX_OUT_TX", "значение": "2"}, {"параметр": "PAYER_TARGET_MIN_IN_DEG", "значение": "5"}, {"параметр": "PRIORITY_WEIGHTS", "значение": "{\"role\": 0.3, \"money\": 0.3, \"brokerage\": 0.2, \"volume\": 0.1, \"temporal\": 0.1}"}, {"параметр": "RANDOM_SEED", "значение": "42"}, {"параметр": "ROLE_WEIGHT", "значение": "{\"coordinator\": 1.0, \"consolidator\": 0.8, \"distributor\": 0.7, \"transit\": 0.5, \"terminal\": 0.3, \"peripheral\": 0.1, \"payer\": 0.05}"}, {"параметр": "SYNC_MIN_PAYERS", "значение": "3"}, {"параметр": "TERMINAL_PT_MAX", "значение": "0.1"}, {"параметр": "TOP_N", "значение": "30"}, {"параметр": "TRANSIT_PT", "значение": "[0.8, 1.2]"}, {"параметр": "TRUNC_TERMINAL_MIN_P", "значение": "0.6"}]</t>
+          <t>[{"параметр": "AGG_MAX_HHI", "значение": "0.15"}, {"параметр": "AGG_MIN_ACTIVE_DAYS", "значение": "12"}, {"параметр": "AGG_MIN_IN_DEG", "значение": "10"}, {"параметр": "AGG_MIN_ONE_OFF", "значение": "0.8"}, {"параметр": "AMBIGUOUS_MARGIN", "значение": "0.1"}, {"параметр": "CHRONO_GAPS", "значение": "{\"any\": 31, \"7d\": 7, \"2d\": 2}"}, {"параметр": "CONF_LEVELS", "значение": "[0.5, 0.75]"}, {"параметр": "CONS_MIN_IN_DEG", "значение": "5"}, {"параметр": "COORD_MIN_KEY_LINKS", "значение": "3"}, {"параметр": "DIST_MIN_OUT_DEG", "значение": "10"}, {"параметр": "EXT_FUNDING_MAX_TRACKED_OUT", "значение": "0.1"}, {"параметр": "EXT_FUNDING_PT", "значение": "2.0"}, {"параметр": "FAST_DAYS", "значение": "2"}, {"параметр": "HHI_DOMINANT", "значение": "0.5"}, {"параметр": "MULT", "значение": "{\"no_chrono\": 0.5, \"external_funding\": 0.7, \"seed\": 0.6, \"seed_above_bottom\": 0.8, \"payer\": 0.2, \"excluded\": 0.0}"}, {"параметр": "NEAR_THRESHOLD", "значение": "[5000, 7000]"}, {"параметр": "PATH_GAP_DAYS", "значение": "7"}, {"параметр": "PAYER_MAX_KZT", "значение": "100000"}, {"параметр": "PAYER_MAX_OUT_DEG", "значение": "2"}, {"параметр": "PAYER_MAX_OUT_TX", "значение": "2"}, {"параметр": "PAYER_TARGET_MIN_IN_DEG", "значение": "5"}, {"параметр": "PRIORITY_WEIGHTS", "значение": "{\"role\": 0.3, \"money\": 0.3, \"brokerage\": 0.2, \"volume\": 0.1, \"temporal\": 0.1}"}, {"параметр": "RANDOM_SEED", "значение": "42"}, {"параметр": "RANDOM_TRIALS", "значение": "100"}, {"параметр": "ROLE_WEIGHT", "значение": "{\"coordinator\": 1.0, \"consolidator\": 0.8, \"distributor\": 0.7, \"transit\": 0.5, \"terminal\": 0.3, \"peripheral\": 0.1, \"payer\": 0.05}"}, {"параметр": "SYNC_MIN_PAYERS", "значение": "3"}, {"параметр": "TERMINAL_PT_MAX", "значение": "0.1"}, {"параметр": "TOP_N", "значение": "30"}, {"параметр": "TRANSIT_PT", "значение": "[0.8, 1.2]"}, {"параметр": "TRUNC_TERMINAL_MIN_P", "значение": "0.6"}]</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
@@ -23464,14 +23488,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
-    <col width="39" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -23514,7 +23538,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Комбинация входящих/исходящих либо связей с ключевыми узлами; COORD_MIN_KEY_LINKS</t>
+          <t>(in_deg ≥ 5 и out_deg ≥ 10) или (from_key ≥ 3 и to_key ≥ 3); key — узлы, прошедшие ворота consolidator, distributor или transit</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -23524,7 +23548,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>docs/TEAM_PLAN.md §7.2 (спецификация)</t>
+          <t>graf.roles: правила; graf.config: текущие пороги</t>
         </is>
       </c>
     </row>
@@ -23541,7 +23565,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Число плательщиков ≥ CONS_MIN_IN_DEG</t>
+          <t>in_deg ≥ 5</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -23551,7 +23575,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>docs/TEAM_PLAN.md §7.2 (спецификация)</t>
+          <t>graf.roles: правила; graf.config: текущие пороги</t>
         </is>
       </c>
     </row>
@@ -23568,7 +23592,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Число получателей ≥ DIST_MIN_OUT_DEG</t>
+          <t>out_deg ≥ 10</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -23578,7 +23602,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>docs/TEAM_PLAN.md §7.2 (спецификация)</t>
+          <t>graf.roles: правила; graf.config: текущие пороги</t>
         </is>
       </c>
     </row>
@@ -23595,21 +23619,21 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Не seed, есть вход/выход, pass_through в TRANSIT_PT</t>
+          <t>не seed; in_deg ≥ 1; out_deg ≥ 1; 0.8 ≤ pass_through ≤ 1.2</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>0.5·(1-|1-pt|/0.2)+0.3·fast_out_share+0.2·[seed_exp_chrono&gt;0]</t>
+          <t>0.5·max(0,1−|1−pass_through|/0.2)+0.3·fast_out_share+0.2·[seed_exp_chrono&gt;0]</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>docs/TEAM_PLAN.md §7.2 (спецификация)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>graf.roles: правила; graf.config: текущие пороги</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>terminal</t>
@@ -23622,17 +23646,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Наблюдаемый выход: out=0 или pt&lt;TERMINAL_PT_MAX; на границе — оценка по p_forward</t>
+          <t>depth ≤ 3; in_deg ≥ 1; (out_deg = 0 или (не seed и pass_through &lt; 0.1)); иначе оценка на depth = 4 при 1−p_forward ≥ 0.6, если не выбрана другая роль</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>0.7+0.3·tracked_share_in; на границе: 1-p_forward</t>
+          <t>0.7+0.3·tracked_share_in; оценка на depth=4: 1−p_forward</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>docs/TEAM_PLAN.md §7.2 (спецификация)</t>
+          <t>graf.roles: правила; graf.config: текущие пороги</t>
         </is>
       </c>
     </row>
@@ -23659,7 +23683,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>docs/TEAM_PLAN.md §7.2 (спецификация)</t>
+          <t>graf.roles: правила; graf.config: текущие пороги</t>
         </is>
       </c>
     </row>
@@ -23676,7 +23700,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Не seed; мало исходящих и небольшая сумма; получатель с большим входом; не транзит</t>
+          <t>не seed; out_deg ≤ 2; out_tx ≤ 2; out_kzt ≤ 100000; хотя бы один получатель с in_deg ≥ 5; ворота transit не пройдены</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -23686,39 +23710,43 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>docs/TEAM_PLAN.md §7.2 (спецификация)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
+          <t>graf.roles: правила; graf.config: текущие пороги</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>AGG_MAX_HHI</t>
+          <t>Порядок выбора</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr"/>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>0.15</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
+          <t>coordinator → payer → максимальный скор среди consolidator/distributor/transit/terminal с пройденными воротами → terminal (оценка на depth=4) → peripheral</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Скор выбранной роли; у seed pass_through не определяет роль. Скоры эвристические, не вероятности вины.</t>
+        </is>
+      </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>graf.config: текущие параметры</t>
+          <t>graf.roles.assign_roles</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>AGG_MIN_ACTIVE_DAYS</t>
+          <t>AGG_MAX_HHI</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -23731,13 +23759,13 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>AGG_MIN_IN_DEG</t>
+          <t>AGG_MIN_ACTIVE_DAYS</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -23750,13 +23778,13 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>AGG_MIN_ONE_OFF</t>
+          <t>AGG_MIN_IN_DEG</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -23769,13 +23797,13 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>AMBIGUOUS_MARGIN</t>
+          <t>AGG_MIN_ONE_OFF</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -23788,13 +23816,13 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>CHRONO_GAPS</t>
+          <t>AMBIGUOUS_MARGIN</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>{"any": 31, "7d": 7, "2d": 2}</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -23807,13 +23835,13 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CONF_LEVELS</t>
+          <t>CHRONO_GAPS</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr"/>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>[0.5, 0.75]</t>
+          <t>{"any": 31, "7d": 7, "2d": 2}</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
@@ -23826,13 +23854,13 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>CONS_MIN_IN_DEG</t>
+          <t>CONF_LEVELS</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>[0.5, 0.75]</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
@@ -23845,13 +23873,13 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>COORD_MIN_KEY_LINKS</t>
+          <t>CONS_MIN_IN_DEG</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr"/>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -23864,13 +23892,13 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DIST_MIN_OUT_DEG</t>
+          <t>COORD_MIN_KEY_LINKS</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
@@ -23883,13 +23911,13 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>EXT_FUNDING_MAX_TRACKED_OUT</t>
+          <t>DIST_MIN_OUT_DEG</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
@@ -23902,13 +23930,13 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>EXT_FUNDING_PT</t>
+          <t>EXT_FUNDING_MAX_TRACKED_OUT</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr"/>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
@@ -23921,13 +23949,13 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>FAST_DAYS</t>
+          <t>EXT_FUNDING_PT</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
@@ -23940,13 +23968,13 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>HHI_DOMINANT</t>
+          <t>FAST_DAYS</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -23959,13 +23987,13 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>MULT</t>
+          <t>HHI_DOMINANT</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>{"no_chrono": 0.5, "external_funding": 0.7, "seed": 0.6, "seed_above_bottom": 0.8, "payer": 0.2, "excluded": 0.0}</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
@@ -23978,13 +24006,13 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>NEAR_THRESHOLD</t>
+          <t>MULT</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>[5000, 7000]</t>
+          <t>{"no_chrono": 0.5, "external_funding": 0.7, "seed": 0.6, "seed_above_bottom": 0.8, "payer": 0.2, "excluded": 0.0}</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
@@ -23997,13 +24025,13 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>PATH_GAP_DAYS</t>
+          <t>NEAR_THRESHOLD</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>[5000, 7000]</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
@@ -24016,13 +24044,13 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>PAYER_MAX_KZT</t>
+          <t>PATH_GAP_DAYS</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>100000</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
@@ -24035,13 +24063,13 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>PAYER_MAX_OUT_DEG</t>
+          <t>PAYER_MAX_KZT</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>100000</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
@@ -24054,7 +24082,7 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>PAYER_MAX_OUT_TX</t>
+          <t>PAYER_MAX_OUT_DEG</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr"/>
@@ -24073,13 +24101,13 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>PAYER_TARGET_MIN_IN_DEG</t>
+          <t>PAYER_MAX_OUT_TX</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr"/>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr"/>
@@ -24092,13 +24120,13 @@
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>PRIORITY_WEIGHTS</t>
+          <t>PAYER_TARGET_MIN_IN_DEG</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>{"role": 0.3, "money": 0.3, "brokerage": 0.2, "volume": 0.1, "temporal": 0.1}</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr"/>
@@ -24111,13 +24139,13 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>RANDOM_SEED</t>
+          <t>PRIORITY_WEIGHTS</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>{"role": 0.3, "money": 0.3, "brokerage": 0.2, "volume": 0.1, "temporal": 0.1}</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr"/>
@@ -24130,13 +24158,13 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ROLE_WEIGHT</t>
+          <t>RANDOM_SEED</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr"/>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>{"coordinator": 1.0, "consolidator": 0.8, "distributor": 0.7, "transit": 0.5, "terminal": 0.3, "peripheral": 0.1, "payer": 0.05}</t>
+          <t>42</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr"/>
@@ -24149,13 +24177,13 @@
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>SYNC_MIN_PAYERS</t>
+          <t>RANDOM_TRIALS</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr"/>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>100</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr"/>
@@ -24168,13 +24196,13 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>TERMINAL_PT_MAX</t>
+          <t>ROLE_WEIGHT</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>{"coordinator": 1.0, "consolidator": 0.8, "distributor": 0.7, "transit": 0.5, "terminal": 0.3, "peripheral": 0.1, "payer": 0.05}</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr"/>
@@ -24187,13 +24215,13 @@
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>TOP_N</t>
+          <t>SYNC_MIN_PAYERS</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr"/>
@@ -24206,13 +24234,13 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>TRANSIT_PT</t>
+          <t>TERMINAL_PT_MAX</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>[0.8, 1.2]</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr"/>
@@ -24225,13 +24253,13 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>TRUNC_TERMINAL_MIN_P</t>
+          <t>TOP_N</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr"/>
@@ -24241,8 +24269,46 @@
         </is>
       </c>
     </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>TRANSIT_PT</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>[0.8, 1.2]</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>graf.config: текущие параметры</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>TRUNC_TERMINAL_MIN_P</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>graf.config: текущие параметры</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E37"/>
+  <autoFilter ref="A1:E39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24253,13 +24319,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="47" customWidth="1" min="4" max="4"/>
+    <col width="57" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -25166,8 +25232,3858 @@
         </is>
       </c>
     </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>100000008546855100</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>100000005456919100</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>100000008438656100</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>100000004692798100</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>100000006111439100</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>75% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>100000006901046100</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>100000008501413100</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>100000005661829100</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>100000005287097100</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>57% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>100000003035737100</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>100000007939160100</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>100000004186824100</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>100000007593823100</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>67% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>100000004180097100</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>71% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>100000004816564100</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>100000003809101100</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>100000001746925100</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>100000008582730100</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>100000006443391100</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="30" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>100000003684369100</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>100000003068941100</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="30" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>100000003246024100</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="30" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>100000000831684100</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>67% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="30" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>100000000343175100</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="30" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>100000004386331100</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>100000004221668100</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>100000005602999100</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>100000005124479100</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>100000005168487100</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>71% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="30" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>100000008169544100</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>86% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>100000007322059100</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>100000008443341100</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="30" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>100000004544958100</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="30" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>100000005619339100</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="30" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>100000005382566100</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>100000006714366100</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="30" customHeight="1">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>100000001049200100</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>80% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="30" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>100000006225798100</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="30" customHeight="1">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>100000003016635100</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="30" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>100000006385877100</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>60% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="30" customHeight="1">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>100000006866783100</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="30" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>100000001616816100</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="30" customHeight="1">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>100000005022552100</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="30" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>100000008637537100</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="30" customHeight="1">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>100000001732159100</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>100000000926766100</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="30" customHeight="1">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>100000001373265100</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="30" customHeight="1">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>100000003152964100</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="30" customHeight="1">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>100000001252290100</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="30" customHeight="1">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>100000004765639100</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="30" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>100000005140601100</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>60% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="30" customHeight="1">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>100000002580377100</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="30" customHeight="1">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>100000002904919100</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="30" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>100000004622227100</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="30" customHeight="1">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>100000004698193100</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>80% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="30" customHeight="1">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>100000004552204100</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="30" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>100000008418835100</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="30" customHeight="1">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>100000008314203100</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="30" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>100000004019124100</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="30" customHeight="1">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>100000005911352100</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>67% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="30" customHeight="1">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>100000003188607100</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="30" customHeight="1">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>100000008516839100</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="30" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>100000004467157100</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="30" customHeight="1">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>100000002692750100</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>75% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="30" customHeight="1">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>100000008650785100</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="30" customHeight="1">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>100000002527114100</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="30" customHeight="1">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>100000005523088100</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="30" customHeight="1">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>100000005668605100</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="30" customHeight="1">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>100000008761219100</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="30" customHeight="1">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>100000005493505100</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="30" customHeight="1">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>100000004041163100</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="30" customHeight="1">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>100000002938501100</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="30" customHeight="1">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>100000003977183100</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="30" customHeight="1">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>100000008571433100</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="30" customHeight="1">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>100000008673001100</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="30" customHeight="1">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>100000005519347100</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="30" customHeight="1">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>100000004975919100</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="30" customHeight="1">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>100000005171642100</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="30" customHeight="1">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>100000008659445100</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="30" customHeight="1">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>100000003975102100</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="30" customHeight="1">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>100000005834479100</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="30" customHeight="1">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>100000008601794100</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="30" customHeight="1">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>100000003561031100</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="30" customHeight="1">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>100000001677389100</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="30" customHeight="1">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>100000008579978100</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="30" customHeight="1">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>100000000580561100</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="30" customHeight="1">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>100000007747786100</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="30" customHeight="1">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>100000005498992100</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="30" customHeight="1">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>100000006912294100</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="30" customHeight="1">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>100000008680731100</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="30" customHeight="1">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>100000008738325100</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="30" customHeight="1">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>100000004358004100</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="30" customHeight="1">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>100000004007116100</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="30" customHeight="1">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>100000004971871100</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="30" customHeight="1">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>100000004971871100</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="30" customHeight="1">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>100000004770073100</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="30" customHeight="1">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>100000005367445100</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="30" customHeight="1">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>100000005454368100</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="30" customHeight="1">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>100000006232815100</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="30" customHeight="1">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>100000004368189100</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="30" customHeight="1">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>100000001429930100</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="30" customHeight="1">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>100000005370580100</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="30" customHeight="1">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>100000004193835100</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="30" customHeight="1">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>100000004193835100</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="30" customHeight="1">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>100000005395727100</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="30" customHeight="1">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>100000005077484100</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="30" customHeight="1">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>100000001279272100</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="30" customHeight="1">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>100000003054328100</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="30" customHeight="1">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>100000004097972100</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="30" customHeight="1">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>100000008379273100</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="30" customHeight="1">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>100000005386383100</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="30" customHeight="1">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>100000005409680100</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="30" customHeight="1">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>100000006994985100</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="30" customHeight="1">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>100000007982728100</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="30" customHeight="1">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>100000004269433100</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="30" customHeight="1">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>100000005233755100</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="30" customHeight="1">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>100000003934614100</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="30" customHeight="1">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>100000001415126100</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="30" customHeight="1">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>100000004388983100</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="30" customHeight="1">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>100000003484058100</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="30" customHeight="1">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>100000004813068100</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="30" customHeight="1">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>100000005485830100</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="30" customHeight="1">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>100000001740277100</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="30" customHeight="1">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>100000007018630100</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="30" customHeight="1">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>100000003677936100</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="30" customHeight="1">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>100000008522127100</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="30" customHeight="1">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>100000005264990100</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="30" customHeight="1">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>100000005417257100</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="30" customHeight="1">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>100000004723755100</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="30" customHeight="1">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>100000006249740100</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="30" customHeight="1">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>100000008575624100</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="30" customHeight="1">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>100000008104567100</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="30" customHeight="1">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>100000005392290100</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="30" customHeight="1">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>100000004508696100</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="30" customHeight="1">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>100000008654653100</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="30" customHeight="1">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>100000005744674100</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="30" customHeight="1">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>100000008599354100</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="30" customHeight="1">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>100000004714705100</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="30" customHeight="1">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>100000002916006100</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="30" customHeight="1">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>100000003200071100</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="30" customHeight="1">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>100000008655779100</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="30" customHeight="1">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>100000000806727100</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="30" customHeight="1">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>100000006831291100</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="30" customHeight="1">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>100000006831291100</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="30" customHeight="1">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>100000004071070100</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="30" customHeight="1">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>100000005413948100</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="30" customHeight="1">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>100000005543136100</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="30" customHeight="1">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>100000008686247100</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="30" customHeight="1">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>100000001490461100</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="30" customHeight="1">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>100000000456947100</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="30" customHeight="1">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>100000003265658100</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="30" customHeight="1">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="inlineStr">
+        <is>
+          <t>100000003349739100</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" ht="30" customHeight="1">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>100000003770083100</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="30" customHeight="1">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>100000004021459100</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="30" customHeight="1">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>100000004174835100</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="30" customHeight="1">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>100000005017150100</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="30" customHeight="1">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>100000005087431100</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" ht="30" customHeight="1">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>100000005235389100</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" ht="30" customHeight="1">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>100000005480435100</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" ht="30" customHeight="1">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>100000005495722100</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="30" customHeight="1">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>100000005550592100</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" ht="30" customHeight="1">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>100000005560900100</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" ht="30" customHeight="1">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>100000005568407100</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="30" customHeight="1">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>100000008117324100</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" ht="30" customHeight="1">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>100000008205000100</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" ht="30" customHeight="1">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>100000008513251100</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" ht="30" customHeight="1">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>100000008669037100</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" ht="30" customHeight="1">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>запросить входящие переводы</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>100000008701222100</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>seed: входящие за пределами исходящей выгрузки не видны</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="30" customHeight="1">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>100000002696152100</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="214" ht="30" customHeight="1">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>100000008680912100</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>100% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" ht="30" customHeight="1">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>100000008619857100</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="30" customHeight="1">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>100000004450649100</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" ht="30" customHeight="1">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>100000004629688100</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="30" customHeight="1">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="inlineStr">
+        <is>
+          <t>100000007689942100</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="30" customHeight="1">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>запрос</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>запросить переводы &lt; 5 000 ₸</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>100000003951827100</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>50% исходящих в интервале 5–7 тыс. ₸</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D44"/>
+  <autoFilter ref="A1:D219"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>